<commit_message>
data: backfill FY Summary across all 126 per-stock financials.xlsx
Regenerated every existing per-stock financials.xlsx via
yfinance_fundamentals.py so each carries the new formula-driven FY Summary
tab (FY-3/FY-2/FY-1/TTM, GAAP) and a quarterly balance sheet. Done with 6
bounded-concurrency subagents (rate-limited yfinance), each a serial,
throttled slice. 127/127 now have FY Summary; 0 empty workbooks.

Net-cash names (AMD, ARM, ANET, CRWD, PLTR, SNOW, ASML, TSM, …) show a
blank Net debt row, REIT DLR a blank Capex, and pre-revenue names (NNE,
OKLO, POET) a blank Gross profit — correct graceful degradation (the
line-item isn't in yfinance), flagged in each workbook's Data flags.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/per-stock/AAON/financials.xlsx
+++ b/per-stock/AAON/financials.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income stmt (annual)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income stmt (quarterly)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance sheet (annual)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash flow (annual)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash flow (quarterly)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data flags" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="FY Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Income stmt (annual)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Income stmt (quarterly)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Balance sheet (annual)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Balance sheet (quarterly)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Cash flow (annual)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Cash flow (quarterly)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Data flags" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +24,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -61,11 +67,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -531,7 +540,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10863130624</v>
+        <v>11198969856</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -546,7 +555,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>11306449920</v>
+        <v>11642288128</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -561,7 +570,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>93.39436000000001</v>
+        <v>96.28169</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -576,7 +585,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>40.285538</v>
+        <v>41.530983</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -591,7 +600,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>6.7182517</v>
+        <v>6.92595</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -711,11 +720,11 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-215134368</v>
+        <v>-183581000</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>yfinance info.freeCashflow</t>
+          <t>statement: TTM OCF - |capex| (yfinance quarterly_cashflow)</t>
         </is>
       </c>
     </row>
@@ -741,7 +750,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>132.62</v>
+        <v>136.72</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -785,6 +794,477 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Fiscal-year summary (GAAP, $ except where noted)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>FY-3</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>FY-2</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>FY-1</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>TTM</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Source / formula</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Fiscal period end</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2023-12-31</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>TTM → 2026-03-31</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>annual statement headers; TTM = Σ last 4 quarters</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B3" s="3">
+        <f>'Income stmt (annual)'!D51</f>
+        <v/>
+      </c>
+      <c r="C3" s="3">
+        <f>'Income stmt (annual)'!C51</f>
+        <v/>
+      </c>
+      <c r="D3" s="3">
+        <f>'Income stmt (annual)'!B51</f>
+        <v/>
+      </c>
+      <c r="E3" s="3">
+        <f>SUM('Income stmt (quarterly)'!B48:E48)</f>
+        <v/>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Total Revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Gross profit</t>
+        </is>
+      </c>
+      <c r="B4" s="3">
+        <f>'Income stmt (annual)'!D49</f>
+        <v/>
+      </c>
+      <c r="C4" s="3">
+        <f>'Income stmt (annual)'!C49</f>
+        <v/>
+      </c>
+      <c r="D4" s="3">
+        <f>'Income stmt (annual)'!B49</f>
+        <v/>
+      </c>
+      <c r="E4" s="3">
+        <f>SUM('Income stmt (quarterly)'!B46:E46)</f>
+        <v/>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Gross Profit (GAAP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Gross margin %</t>
+        </is>
+      </c>
+      <c r="B5" s="4">
+        <f>IFERROR(B4/B3,"")</f>
+        <v/>
+      </c>
+      <c r="C5" s="4">
+        <f>IFERROR(C4/C3,"")</f>
+        <v/>
+      </c>
+      <c r="D5" s="4">
+        <f>IFERROR(D4/D3,"")</f>
+        <v/>
+      </c>
+      <c r="E5" s="4">
+        <f>IFERROR(E4/E3,"")</f>
+        <v/>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>GAAP = gross profit / revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Operating income</t>
+        </is>
+      </c>
+      <c r="B6" s="3">
+        <f>'Income stmt (annual)'!D38</f>
+        <v/>
+      </c>
+      <c r="C6" s="3">
+        <f>'Income stmt (annual)'!C38</f>
+        <v/>
+      </c>
+      <c r="D6" s="3">
+        <f>'Income stmt (annual)'!B38</f>
+        <v/>
+      </c>
+      <c r="E6" s="3">
+        <f>SUM('Income stmt (quarterly)'!B36:E36)</f>
+        <v/>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Operating Income</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Operating margin %</t>
+        </is>
+      </c>
+      <c r="B7" s="4">
+        <f>IFERROR(B6/B3,"")</f>
+        <v/>
+      </c>
+      <c r="C7" s="4">
+        <f>IFERROR(C6/C3,"")</f>
+        <v/>
+      </c>
+      <c r="D7" s="4">
+        <f>IFERROR(D6/D3,"")</f>
+        <v/>
+      </c>
+      <c r="E7" s="4">
+        <f>IFERROR(E6/E3,"")</f>
+        <v/>
+      </c>
+      <c r="F7">
+        <f> operating income / revenue</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B8" s="3">
+        <f>'Income stmt (annual)'!D10</f>
+        <v/>
+      </c>
+      <c r="C8" s="3">
+        <f>'Income stmt (annual)'!C10</f>
+        <v/>
+      </c>
+      <c r="D8" s="3">
+        <f>'Income stmt (annual)'!B10</f>
+        <v/>
+      </c>
+      <c r="E8" s="3">
+        <f>SUM('Income stmt (quarterly)'!B10:E10)</f>
+        <v/>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Free cash flow</t>
+        </is>
+      </c>
+      <c r="B9" s="3">
+        <f>'Cash flow (annual)'!D2</f>
+        <v/>
+      </c>
+      <c r="C9" s="3">
+        <f>'Cash flow (annual)'!C2</f>
+        <v/>
+      </c>
+      <c r="D9" s="3">
+        <f>'Cash flow (annual)'!B2</f>
+        <v/>
+      </c>
+      <c r="E9" s="3">
+        <f>SUM('Cash flow (quarterly)'!B2:E2)</f>
+        <v/>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>FCF = OCF − capex</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>FCF margin %</t>
+        </is>
+      </c>
+      <c r="B10" s="4">
+        <f>IFERROR(B9/B3,"")</f>
+        <v/>
+      </c>
+      <c r="C10" s="4">
+        <f>IFERROR(C9/C3,"")</f>
+        <v/>
+      </c>
+      <c r="D10" s="4">
+        <f>IFERROR(D9/D3,"")</f>
+        <v/>
+      </c>
+      <c r="E10" s="4">
+        <f>IFERROR(E9/E3,"")</f>
+        <v/>
+      </c>
+      <c r="F10">
+        <f> FCF / revenue</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Capex</t>
+        </is>
+      </c>
+      <c r="B11" s="3">
+        <f>-'Cash flow (annual)'!D6</f>
+        <v/>
+      </c>
+      <c r="C11" s="3">
+        <f>-'Cash flow (annual)'!C6</f>
+        <v/>
+      </c>
+      <c r="D11" s="3">
+        <f>-'Cash flow (annual)'!B6</f>
+        <v/>
+      </c>
+      <c r="E11" s="3">
+        <f>-SUM('Cash flow (quarterly)'!B6:E6)</f>
+        <v/>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Capex (shown positive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Capex / revenue %</t>
+        </is>
+      </c>
+      <c r="B12" s="4">
+        <f>IFERROR(B11/B3,"")</f>
+        <v/>
+      </c>
+      <c r="C12" s="4">
+        <f>IFERROR(C11/C3,"")</f>
+        <v/>
+      </c>
+      <c r="D12" s="4">
+        <f>IFERROR(D11/D3,"")</f>
+        <v/>
+      </c>
+      <c r="E12" s="4">
+        <f>IFERROR(E11/E3,"")</f>
+        <v/>
+      </c>
+      <c r="F12">
+        <f> capex / revenue</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Net debt</t>
+        </is>
+      </c>
+      <c r="B13" s="3">
+        <f>'Balance sheet (annual)'!D4</f>
+        <v/>
+      </c>
+      <c r="C13" s="3">
+        <f>'Balance sheet (annual)'!C4</f>
+        <v/>
+      </c>
+      <c r="D13" s="3">
+        <f>'Balance sheet (annual)'!B4</f>
+        <v/>
+      </c>
+      <c r="E13" s="3">
+        <f>'Balance sheet (quarterly)'!B4</f>
+        <v/>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Net debt; TTM = MRQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Net debt / EBITDA</t>
+        </is>
+      </c>
+      <c r="B14" s="5">
+        <f>IFERROR(B13/B8,"")</f>
+        <v/>
+      </c>
+      <c r="C14" s="5">
+        <f>IFERROR(C13/C8,"")</f>
+        <v/>
+      </c>
+      <c r="D14" s="5">
+        <f>IFERROR(D13/D8,"")</f>
+        <v/>
+      </c>
+      <c r="E14" s="5">
+        <f>IFERROR(E13/E8,"")</f>
+        <v/>
+      </c>
+      <c r="F14">
+        <f> net debt / EBITDA</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Share count (period-end, M)</t>
+        </is>
+      </c>
+      <c r="B15" s="6">
+        <f>'Balance sheet (annual)'!D2/1e6</f>
+        <v/>
+      </c>
+      <c r="C15" s="6">
+        <f>'Balance sheet (annual)'!C2/1e6</f>
+        <v/>
+      </c>
+      <c r="D15" s="6">
+        <f>'Balance sheet (annual)'!B2/1e6</f>
+        <v/>
+      </c>
+      <c r="E15" s="6">
+        <f>'Balance sheet (quarterly)'!B2/1e6</f>
+        <v/>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>shares ÷ 1e6; TTM = MRQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Share count YoY %</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr"/>
+      <c r="C16" s="4">
+        <f>IFERROR(C15/B15-1,"")</f>
+        <v/>
+      </c>
+      <c r="D16" s="4">
+        <f>IFERROR(D15/C15-1,"")</f>
+        <v/>
+      </c>
+      <c r="E16" s="4">
+        <f>IFERROR(E15/D15-1,"")</f>
+        <v/>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>vs prior period</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1840,7 +2320,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3004,7 +3484,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4554,7 +5034,1843 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H75"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Line item</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>2025-09-30</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>2025-06-30</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>2024-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ordinary Shares Number</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>81851483</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>81691075</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>81593092</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>81509387</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>81348131</v>
+      </c>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Share Issued</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>81851483</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>81691075</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>81593092</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>81509387</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>81348131</v>
+      </c>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Net Debt</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>432676000</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>405842000</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>359101000</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>317263000</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>251423000</v>
+      </c>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Total Debt</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>450867000</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>424646000</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>377947000</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>335778000</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>267830000</v>
+      </c>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tangible Book Value</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>762296000</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>729186000</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>699224000</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>670439000</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>655239000</v>
+      </c>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Invested Capital</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>1366898000</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>1300840000</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>1223252000</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>1150023000</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>1068269000</v>
+      </c>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Working Capital</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>584066000</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>538325000</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>509150000</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>443425000</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>365127000</v>
+      </c>
+      <c r="G8" s="3" t="n"/>
+      <c r="H8" s="3" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Net Tangible Assets</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>762296000</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>729186000</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>699224000</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>670439000</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>655239000</v>
+      </c>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Capital Lease Obligations</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>18178000</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>18791000</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>17805000</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>18501000</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>15413000</v>
+      </c>
+      <c r="G10" s="3" t="n"/>
+      <c r="H10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Common Stock Equity</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>934209000</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>894985000</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>863110000</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>832746000</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>815852000</v>
+      </c>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Total Capitalization</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>1359363000</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>1293305000</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>1223252000</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>1150023000</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>1052269000</v>
+      </c>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Total Equity Gross Minority Interest</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>934209000</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>894985000</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>863110000</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>832746000</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>815852000</v>
+      </c>
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Stockholders Equity</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>934209000</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>894985000</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>863110000</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>832746000</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>815852000</v>
+      </c>
+      <c r="G14" s="3" t="n"/>
+      <c r="H14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Retained Earnings</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>861969000</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>830300000</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>806434000</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>783813000</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>776507000</v>
+      </c>
+      <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Additional Paid In Capital</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>71913000</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>64358000</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>56350000</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>48607000</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>39020000</v>
+      </c>
+      <c r="G16" s="3" t="n"/>
+      <c r="H16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Capital Stock</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>327000</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>327000</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>326000</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>326000</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>325000</v>
+      </c>
+      <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Common Stock</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>327000</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>327000</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>326000</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>326000</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>325000</v>
+      </c>
+      <c r="G18" s="3" t="n"/>
+      <c r="H18" s="3" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Preferred Stock</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="3" t="n"/>
+      <c r="H19" s="3" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Total Liabilities Net Minority Interest</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>855503000</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>791525000</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>670961000</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>566667000</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>484341000</v>
+      </c>
+      <c r="G20" s="3" t="n"/>
+      <c r="H20" s="3" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Total Non Current Liabilities Net Minority Interest</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>495869000</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>460670000</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>420779000</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>355941000</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>277724000</v>
+      </c>
+      <c r="G21" s="3" t="n"/>
+      <c r="H21" s="3" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Other Non Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>12213000</v>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>7770000</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>7303000</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>6824000</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>7043000</v>
+      </c>
+      <c r="G22" s="3" t="n"/>
+      <c r="H22" s="3" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Tradeand Other Payables Non Current</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>8778000</v>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>8738000</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>16233000</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>16193000</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>16153000</v>
+      </c>
+      <c r="G23" s="3" t="n"/>
+      <c r="H23" s="3" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Non Current Deferred Liabilities</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>34899000</v>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>30313000</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>22199000</v>
+      </c>
+      <c r="E24" s="3" t="n"/>
+      <c r="F24" s="3" t="n">
+        <v>5140000</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="3" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Non Current Deferred Taxes Liabilities</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>34899000</v>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>30313000</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>22199000</v>
+      </c>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n">
+        <v>5140000</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="3" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Long Term Debt And Capital Lease Obligation</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>439979000</v>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>413849000</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>375044000</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>332924000</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>249388000</v>
+      </c>
+      <c r="G26" s="3" t="n"/>
+      <c r="H26" s="3" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Long Term Capital Lease Obligation</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>14825000</v>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>15529000</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>14902000</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>15647000</v>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>12971000</v>
+      </c>
+      <c r="G27" s="3" t="n"/>
+      <c r="H27" s="3" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Long Term Debt</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>425154000</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>398320000</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>360142000</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>317277000</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>236417000</v>
+      </c>
+      <c r="G28" s="3" t="n"/>
+      <c r="H28" s="3" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>359634000</v>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>330855000</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>250182000</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>210726000</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>206617000</v>
+      </c>
+      <c r="G29" s="3" t="n"/>
+      <c r="H29" s="3" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Current Deferred Liabilities</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>57335000</v>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>87526000</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>24007000</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>37233000</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>21657000</v>
+      </c>
+      <c r="G30" s="3" t="n"/>
+      <c r="H30" s="3" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Current Deferred Revenue</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>57335000</v>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>87526000</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>24007000</v>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>37233000</v>
+      </c>
+      <c r="F31" s="3" t="n">
+        <v>21657000</v>
+      </c>
+      <c r="G31" s="3" t="n"/>
+      <c r="H31" s="3" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Current Debt And Capital Lease Obligation</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>10888000</v>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>10797000</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>2903000</v>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>2854000</v>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>18442000</v>
+      </c>
+      <c r="G32" s="3" t="n"/>
+      <c r="H32" s="3" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Current Capital Lease Obligation</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>3353000</v>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>3262000</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>2903000</v>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>2854000</v>
+      </c>
+      <c r="F33" s="3" t="n">
+        <v>2442000</v>
+      </c>
+      <c r="G33" s="3" t="n"/>
+      <c r="H33" s="3" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Current Debt</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>7535000</v>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>7535000</v>
+      </c>
+      <c r="D34" s="3" t="n"/>
+      <c r="E34" s="3" t="n"/>
+      <c r="F34" s="3" t="n">
+        <v>16000000</v>
+      </c>
+      <c r="G34" s="3" t="n">
+        <v>16000000</v>
+      </c>
+      <c r="H34" s="3" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Other Current Borrowings</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>7535000</v>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>7535000</v>
+      </c>
+      <c r="D35" s="3" t="n"/>
+      <c r="E35" s="3" t="n"/>
+      <c r="F35" s="3" t="n">
+        <v>16000000</v>
+      </c>
+      <c r="G35" s="3" t="n">
+        <v>16000000</v>
+      </c>
+      <c r="H35" s="3" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Pensionand Other Post Retirement Benefit Plans Current</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>22553000</v>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>19268000</v>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>18721000</v>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>16117000</v>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>16253000</v>
+      </c>
+      <c r="G36" s="3" t="n"/>
+      <c r="H36" s="3" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Payables And Accrued Expenses</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>268858000</v>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>213264000</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>204551000</v>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>154522000</v>
+      </c>
+      <c r="F37" s="3" t="n">
+        <v>150265000</v>
+      </c>
+      <c r="G37" s="3" t="n"/>
+      <c r="H37" s="3" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Current Accrued Expenses</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>71535000</v>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>72231000</v>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>66408000</v>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>47634000</v>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>52340000</v>
+      </c>
+      <c r="G38" s="3" t="n"/>
+      <c r="H38" s="3" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Payables</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>197323000</v>
+      </c>
+      <c r="C39" s="3" t="n">
+        <v>141033000</v>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>138143000</v>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>106888000</v>
+      </c>
+      <c r="F39" s="3" t="n">
+        <v>97925000</v>
+      </c>
+      <c r="G39" s="3" t="n"/>
+      <c r="H39" s="3" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Other Payable</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>35299000</v>
+      </c>
+      <c r="C40" s="3" t="n">
+        <v>30453000</v>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>23431000</v>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>22197000</v>
+      </c>
+      <c r="F40" s="3" t="n">
+        <v>19181000</v>
+      </c>
+      <c r="G40" s="3" t="n"/>
+      <c r="H40" s="3" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Total Tax Payable</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>1885000</v>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>143000</v>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>4972000</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>3049000</v>
+      </c>
+      <c r="F41" s="3" t="n">
+        <v>1589000</v>
+      </c>
+      <c r="G41" s="3" t="n"/>
+      <c r="H41" s="3" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Income Tax Payable</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>1885000</v>
+      </c>
+      <c r="C42" s="3" t="n">
+        <v>143000</v>
+      </c>
+      <c r="D42" s="3" t="n"/>
+      <c r="E42" s="3" t="n"/>
+      <c r="F42" s="3" t="n"/>
+      <c r="G42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Accounts Payable</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>160139000</v>
+      </c>
+      <c r="C43" s="3" t="n">
+        <v>110437000</v>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>109740000</v>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>81642000</v>
+      </c>
+      <c r="F43" s="3" t="n">
+        <v>77155000</v>
+      </c>
+      <c r="G43" s="3" t="n"/>
+      <c r="H43" s="3" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Total Assets</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>1789712000</v>
+      </c>
+      <c r="C44" s="3" t="n">
+        <v>1686510000</v>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>1534071000</v>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>1399413000</v>
+      </c>
+      <c r="F44" s="3" t="n">
+        <v>1300193000</v>
+      </c>
+      <c r="G44" s="3" t="n"/>
+      <c r="H44" s="3" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Total Non Current Assets</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>846012000</v>
+      </c>
+      <c r="C45" s="3" t="n">
+        <v>817330000</v>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>774739000</v>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>745262000</v>
+      </c>
+      <c r="F45" s="3" t="n">
+        <v>728449000</v>
+      </c>
+      <c r="G45" s="3" t="n"/>
+      <c r="H45" s="3" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Other Non Current Assets</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>1907000</v>
+      </c>
+      <c r="C46" s="3" t="n">
+        <v>2281000</v>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>2151000</v>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>2422000</v>
+      </c>
+      <c r="F46" s="3" t="n">
+        <v>808000</v>
+      </c>
+      <c r="G46" s="3" t="n"/>
+      <c r="H46" s="3" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Non Current Deferred Assets</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n"/>
+      <c r="C47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="3" t="n">
+        <v>3259000</v>
+      </c>
+      <c r="F47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="3" t="n">
+        <v>836000</v>
+      </c>
+      <c r="H47" s="3" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Non Current Deferred Taxes Assets</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n"/>
+      <c r="C48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" s="3" t="n">
+        <v>3259000</v>
+      </c>
+      <c r="F48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="3" t="n">
+        <v>836000</v>
+      </c>
+      <c r="H48" s="3" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Goodwill And Other Intangible Assets</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>171913000</v>
+      </c>
+      <c r="C49" s="3" t="n">
+        <v>165799000</v>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>163886000</v>
+      </c>
+      <c r="E49" s="3" t="n">
+        <v>162307000</v>
+      </c>
+      <c r="F49" s="3" t="n">
+        <v>160613000</v>
+      </c>
+      <c r="G49" s="3" t="n"/>
+      <c r="H49" s="3" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Other Intangible Assets</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>90021000</v>
+      </c>
+      <c r="C50" s="3" t="n">
+        <v>83907000</v>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>81994000</v>
+      </c>
+      <c r="E50" s="3" t="n">
+        <v>80415000</v>
+      </c>
+      <c r="F50" s="3" t="n">
+        <v>78721000</v>
+      </c>
+      <c r="G50" s="3" t="n"/>
+      <c r="H50" s="3" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Goodwill</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>81892000</v>
+      </c>
+      <c r="C51" s="3" t="n">
+        <v>81892000</v>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>81892000</v>
+      </c>
+      <c r="E51" s="3" t="n">
+        <v>81892000</v>
+      </c>
+      <c r="F51" s="3" t="n">
+        <v>81892000</v>
+      </c>
+      <c r="G51" s="3" t="n"/>
+      <c r="H51" s="3" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Net PPE</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>672192000</v>
+      </c>
+      <c r="C52" s="3" t="n">
+        <v>649250000</v>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>608702000</v>
+      </c>
+      <c r="E52" s="3" t="n">
+        <v>577274000</v>
+      </c>
+      <c r="F52" s="3" t="n">
+        <v>567028000</v>
+      </c>
+      <c r="G52" s="3" t="n"/>
+      <c r="H52" s="3" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Accumulated Depreciation</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>-380492000</v>
+      </c>
+      <c r="C53" s="3" t="n">
+        <v>-372515000</v>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>-355826000</v>
+      </c>
+      <c r="E53" s="3" t="n">
+        <v>-338933000</v>
+      </c>
+      <c r="F53" s="3" t="n">
+        <v>-324846000</v>
+      </c>
+      <c r="G53" s="3" t="n"/>
+      <c r="H53" s="3" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Gross PPE</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1052684000</v>
+      </c>
+      <c r="C54" s="3" t="n">
+        <v>1021765000</v>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>964528000</v>
+      </c>
+      <c r="E54" s="3" t="n">
+        <v>916207000</v>
+      </c>
+      <c r="F54" s="3" t="n">
+        <v>891874000</v>
+      </c>
+      <c r="G54" s="3" t="n"/>
+      <c r="H54" s="3" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Other Properties</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>17335000</v>
+      </c>
+      <c r="C55" s="3" t="n">
+        <v>17988000</v>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>17050000</v>
+      </c>
+      <c r="E55" s="3" t="n">
+        <v>17795000</v>
+      </c>
+      <c r="F55" s="3" t="n">
+        <v>14751000</v>
+      </c>
+      <c r="G55" s="3" t="n"/>
+      <c r="H55" s="3" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Machinery Furniture Equipment</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>648835000</v>
+      </c>
+      <c r="C56" s="3" t="n">
+        <v>619710000</v>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>586685000</v>
+      </c>
+      <c r="E56" s="3" t="n">
+        <v>552054000</v>
+      </c>
+      <c r="F56" s="3" t="n">
+        <v>535891000</v>
+      </c>
+      <c r="G56" s="3" t="n"/>
+      <c r="H56" s="3" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Buildings And Improvements</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>369366000</v>
+      </c>
+      <c r="C57" s="3" t="n">
+        <v>366919000</v>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>343645000</v>
+      </c>
+      <c r="E57" s="3" t="n">
+        <v>329210000</v>
+      </c>
+      <c r="F57" s="3" t="n">
+        <v>324084000</v>
+      </c>
+      <c r="G57" s="3" t="n"/>
+      <c r="H57" s="3" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Land And Improvements</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>17148000</v>
+      </c>
+      <c r="C58" s="3" t="n">
+        <v>17148000</v>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>17148000</v>
+      </c>
+      <c r="E58" s="3" t="n">
+        <v>17148000</v>
+      </c>
+      <c r="F58" s="3" t="n">
+        <v>17148000</v>
+      </c>
+      <c r="G58" s="3" t="n"/>
+      <c r="H58" s="3" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Properties</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C59" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="3" t="n"/>
+      <c r="H59" s="3" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Current Assets</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="n">
+        <v>943700000</v>
+      </c>
+      <c r="C60" s="3" t="n">
+        <v>869180000</v>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>759332000</v>
+      </c>
+      <c r="E60" s="3" t="n">
+        <v>654151000</v>
+      </c>
+      <c r="F60" s="3" t="n">
+        <v>571744000</v>
+      </c>
+      <c r="G60" s="3" t="n"/>
+      <c r="H60" s="3" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Other Current Assets</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="n">
+        <v>21177000</v>
+      </c>
+      <c r="C61" s="3" t="n">
+        <v>17921000</v>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>7668000</v>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>6791000</v>
+      </c>
+      <c r="F61" s="3" t="n">
+        <v>9438000</v>
+      </c>
+      <c r="G61" s="3" t="n"/>
+      <c r="H61" s="3" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Restricted Cash</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="n">
+        <v>1087000</v>
+      </c>
+      <c r="C62" s="3" t="n">
+        <v>1226000</v>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>1226000</v>
+      </c>
+      <c r="E62" s="3" t="n">
+        <v>1307000</v>
+      </c>
+      <c r="F62" s="3" t="n">
+        <v>1389000</v>
+      </c>
+      <c r="G62" s="3" t="n"/>
+      <c r="H62" s="3" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Inventory</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="n">
+        <v>313203000</v>
+      </c>
+      <c r="C63" s="3" t="n">
+        <v>261151000</v>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>250511000</v>
+      </c>
+      <c r="E63" s="3" t="n">
+        <v>234980000</v>
+      </c>
+      <c r="F63" s="3" t="n">
+        <v>198852000</v>
+      </c>
+      <c r="G63" s="3" t="n"/>
+      <c r="H63" s="3" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Inventories Adjustments Allowances</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="n">
+        <v>-6045000</v>
+      </c>
+      <c r="C64" s="3" t="n">
+        <v>-5344000</v>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>-6217000</v>
+      </c>
+      <c r="E64" s="3" t="n">
+        <v>-5480000</v>
+      </c>
+      <c r="F64" s="3" t="n">
+        <v>-5249000</v>
+      </c>
+      <c r="G64" s="3" t="n"/>
+      <c r="H64" s="3" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Finished Goods</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="n">
+        <v>511000</v>
+      </c>
+      <c r="C65" s="3" t="n">
+        <v>593000</v>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>971000</v>
+      </c>
+      <c r="E65" s="3" t="n">
+        <v>892000</v>
+      </c>
+      <c r="F65" s="3" t="n">
+        <v>606000</v>
+      </c>
+      <c r="G65" s="3" t="n"/>
+      <c r="H65" s="3" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Work In Process</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="n">
+        <v>1482000</v>
+      </c>
+      <c r="C66" s="3" t="n">
+        <v>475000</v>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>13000</v>
+      </c>
+      <c r="E66" s="3" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F66" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="3" t="n"/>
+      <c r="H66" s="3" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Raw Materials</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="n">
+        <v>317255000</v>
+      </c>
+      <c r="C67" s="3" t="n">
+        <v>265427000</v>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>255744000</v>
+      </c>
+      <c r="E67" s="3" t="n">
+        <v>239564000</v>
+      </c>
+      <c r="F67" s="3" t="n">
+        <v>203495000</v>
+      </c>
+      <c r="G67" s="3" t="n"/>
+      <c r="H67" s="3" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Receivables</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="n">
+        <v>608220000</v>
+      </c>
+      <c r="C68" s="3" t="n">
+        <v>588869000</v>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>498886000</v>
+      </c>
+      <c r="E68" s="3" t="n">
+        <v>411059000</v>
+      </c>
+      <c r="F68" s="3" t="n">
+        <v>361071000</v>
+      </c>
+      <c r="G68" s="3" t="n"/>
+      <c r="H68" s="3" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Other Receivables</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="n">
+        <v>298368000</v>
+      </c>
+      <c r="C69" s="3" t="n">
+        <v>247037000</v>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>207140000</v>
+      </c>
+      <c r="E69" s="3" t="n">
+        <v>233184000</v>
+      </c>
+      <c r="F69" s="3" t="n">
+        <v>188656000</v>
+      </c>
+      <c r="G69" s="3" t="n"/>
+      <c r="H69" s="3" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Taxes Receivable</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="n">
+        <v>19691000</v>
+      </c>
+      <c r="C70" s="3" t="n">
+        <v>27445000</v>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>25508000</v>
+      </c>
+      <c r="E70" s="3" t="n">
+        <v>7302000</v>
+      </c>
+      <c r="F70" s="3" t="n">
+        <v>7438000</v>
+      </c>
+      <c r="G70" s="3" t="n"/>
+      <c r="H70" s="3" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Accounts Receivable</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="n">
+        <v>290161000</v>
+      </c>
+      <c r="C71" s="3" t="n">
+        <v>314387000</v>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>266238000</v>
+      </c>
+      <c r="E71" s="3" t="n">
+        <v>170573000</v>
+      </c>
+      <c r="F71" s="3" t="n">
+        <v>164977000</v>
+      </c>
+      <c r="G71" s="3" t="n"/>
+      <c r="H71" s="3" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Allowance For Doubtful Accounts Receivable</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="n">
+        <v>-1188000</v>
+      </c>
+      <c r="C72" s="3" t="n">
+        <v>-1308000</v>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>-1330000</v>
+      </c>
+      <c r="E72" s="3" t="n">
+        <v>-1308000</v>
+      </c>
+      <c r="F72" s="3" t="n">
+        <v>-1126000</v>
+      </c>
+      <c r="G72" s="3" t="n"/>
+      <c r="H72" s="3" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Gross Accounts Receivable</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="n">
+        <v>291349000</v>
+      </c>
+      <c r="C73" s="3" t="n">
+        <v>315695000</v>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>267568000</v>
+      </c>
+      <c r="E73" s="3" t="n">
+        <v>171881000</v>
+      </c>
+      <c r="F73" s="3" t="n">
+        <v>166103000</v>
+      </c>
+      <c r="G73" s="3" t="n"/>
+      <c r="H73" s="3" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Cash Cash Equivalents And Short Term Investments</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="n">
+        <v>13000</v>
+      </c>
+      <c r="C74" s="3" t="n">
+        <v>13000</v>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>1041000</v>
+      </c>
+      <c r="E74" s="3" t="n">
+        <v>14000</v>
+      </c>
+      <c r="F74" s="3" t="n">
+        <v>994000</v>
+      </c>
+      <c r="G74" s="3" t="n"/>
+      <c r="H74" s="3" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Cash And Cash Equivalents</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="n">
+        <v>13000</v>
+      </c>
+      <c r="C75" s="3" t="n">
+        <v>13000</v>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>1041000</v>
+      </c>
+      <c r="E75" s="3" t="n">
+        <v>14000</v>
+      </c>
+      <c r="F75" s="3" t="n">
+        <v>994000</v>
+      </c>
+      <c r="G75" s="3" t="n"/>
+      <c r="H75" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5792,7 +8108,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7102,7 +9418,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>